<commit_message>
Update multiple template Excel files
</commit_message>
<xml_diff>
--- a/static/templates/asset_type_template.xlsx
+++ b/static/templates/asset_type_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Muttraf\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cydea\grc_backend\static\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D795BD40-7080-4422-9B52-EBC90548F5E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42C7CCF-FDA0-4EF4-A8CF-69064BBA4C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{17C1CE52-05C9-4D28-8FBB-D81BA6FCE39E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{17C1CE52-05C9-4D28-8FBB-D81BA6FCE39E}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -547,9 +547,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -609,9 +610,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -649,7 +650,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -755,7 +756,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -897,7 +898,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -906,16 +907,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BFF5B51-E5AE-44D7-9958-1416F56C2210}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.26171875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.5234375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.26171875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="29.41796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.44140625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -928,11 +929,11 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -945,7 +946,7 @@
       <c r="D2" t="s">
         <v>5</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -958,7 +959,7 @@
           <x14:formula1>
             <xm:f>'Dropdown Options'!#REF!</xm:f>
           </x14:formula1>
-          <xm:sqref>E2:E26 C2:C18</xm:sqref>
+          <xm:sqref>C3:C18 E3:E26</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{44013BF7-80D3-4D5B-AFD4-A13C1D1B34D2}">
           <x14:formula1>
@@ -975,50 +976,50 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5F6FC7C-F41D-423D-93C9-8925280658D3}">
   <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
     </row>
   </sheetData>

</xml_diff>